<commit_message>
Fase 2 v7 (en curso): cambio 1.6, análisis del profesor y supresión complementaria
- Cambio 1.6 del protocolo: H11, H13, H14 y H17a alineadas con la Fase 1 v6.
- Análisis R1 a R5 pedidos por el profesor guía (eda/revision_profesor.py).
- Supresión complementaria (eda/proteccion.py y eda/proteccion_tablas.py):
  ninguna suma conocida queda con una sola celda oculta.
- Documentos de las Fases 1 y 2, Fase 3 (hallazgos RUT) e INCIDENTES sin
  conteos de menos de diez casos.
- El registro de cifras admite «<10» (la configuración se cambia en el
  commit siguiente, después de la corrida de prueba).

Las salidas y el informe Word v7 van en el commit siguiente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192aVCC8aocJbeAsVJ1Mter
</commit_message>
<xml_diff>
--- a/docs/fase2_comprension_datos/Trazabilidad_129_columnas.xlsx
+++ b/docs/fase2_comprension_datos/Trazabilidad_129_columnas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="129 columnas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por grupo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="129 columnas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Por grupo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'129 columnas'!$A$1:$Q$130</definedName>
@@ -2039,11 +2039,15 @@
           <t>Concepto ("servicio/especialidad", condicional)</t>
         </is>
       </c>
-      <c r="G17" s="7" t="n">
-        <v>5.2e-05</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>5.2e-05</v>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>menos de 0,0002 (menos de diez registros)</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>menos de 0,0002 (menos de diez registros)</t>
+        </is>
       </c>
       <c r="I17" s="7" t="n">
         <v>0.00375</v>
@@ -4367,11 +4371,15 @@
           <t>Concepto indirecto (recién nacidos, filtro MDC 15); columnas RN no nombradas</t>
         </is>
       </c>
-      <c r="G53" s="7" t="n">
-        <v>99.999983</v>
-      </c>
-      <c r="H53" s="7" t="n">
-        <v>99.999983</v>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
       </c>
       <c r="I53" s="7" t="n">
         <v>1</v>
@@ -4430,11 +4438,15 @@
           <t>Concepto indirecto (recién nacidos, filtro MDC 15); columnas RN no nombradas</t>
         </is>
       </c>
-      <c r="G54" s="7" t="n">
-        <v>99.999966</v>
-      </c>
-      <c r="H54" s="7" t="n">
-        <v>99.999966</v>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
       </c>
       <c r="I54" s="7" t="n">
         <v>1</v>
@@ -8924,11 +8936,15 @@
           <t>NO MENCIONADA</t>
         </is>
       </c>
-      <c r="G122" s="7" t="n">
-        <v>99.99984499999999</v>
-      </c>
-      <c r="H122" s="7" t="n">
-        <v>99.99984499999999</v>
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
+      </c>
+      <c r="H122" s="7" t="inlineStr">
+        <is>
+          <t>más de 99,9998 (menos de diez registros con dato)</t>
+        </is>
       </c>
       <c r="I122" s="7" t="n">
         <v>1</v>

</xml_diff>